<commit_message>
Final version of the unit description schema.
</commit_message>
<xml_diff>
--- a/CDOP_Unit_Description_Schema.xlsx
+++ b/CDOP_Unit_Description_Schema.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikodem_lacki/Documents/work/Carbon-Data-Open-Protocol/Carbon-Data-Open-Protocol/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F940592-9247-A341-A210-B0196B29E82D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE4635E-1A4D-294A-9A69-1A48ED79ACAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14400" yWindow="-18560" windowWidth="27640" windowHeight="16680" xr2:uid="{91F153D1-A085-9E48-A05D-64480C7AD125}"/>
+    <workbookView xWindow="13420" yWindow="14700" windowWidth="38400" windowHeight="16460" xr2:uid="{91F153D1-A085-9E48-A05D-64480C7AD125}"/>
   </bookViews>
   <sheets>
     <sheet name="Unit Description" sheetId="3" r:id="rId1"/>
+    <sheet name="Unit Type Lookup" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="106">
   <si>
     <t>CDOP_field_label</t>
   </si>
@@ -62,18 +63,12 @@
     <t>CDOP_definition</t>
   </si>
   <si>
-    <t>available for resell</t>
-  </si>
-  <si>
     <t>Unit</t>
   </si>
   <si>
     <t>0..1</t>
   </si>
   <si>
-    <t>boolean</t>
-  </si>
-  <si>
     <t>Optional</t>
   </si>
   <si>
@@ -83,9 +78,6 @@
     <t>Public</t>
   </si>
   <si>
-    <t>Whether the project is open to resellers.</t>
-  </si>
-  <si>
     <t>Text</t>
   </si>
   <si>
@@ -95,9 +87,6 @@
     <t>Required</t>
   </si>
   <si>
-    <t>Issuance</t>
-  </si>
-  <si>
     <t>Integer</t>
   </si>
   <si>
@@ -110,12 +99,6 @@
     <t>Identifier used to track the unit to the original issuance it was part of.</t>
   </si>
   <si>
-    <t>issuance unit count</t>
-  </si>
-  <si>
-    <t>The total number of credits issued by the registry from the start of the project. Complete raw registry issuance tables are available on our GitHub. As of v6, issuance figures do not include buffer pool credits. Issuance figures also do not include Gold Standard planned emissions reductions (PERs) which are ex-ante credits representing expected future reductions. These are summed separately. Note that issued credit totals for VCS include all credits in a vintage if any credits of that vintage have been issued. This is different from how VCS reports issuances (please see the FAQ tab for a more detailed description).</t>
-  </si>
-  <si>
     <t>metric</t>
   </si>
   <si>
@@ -155,9 +138,6 @@
     <t>User Input</t>
   </si>
   <si>
-    <t>unit status reason</t>
-  </si>
-  <si>
     <t>1..*</t>
   </si>
   <si>
@@ -167,18 +147,9 @@
     <t>Select the status that best desribes the current state of the units.</t>
   </si>
   <si>
-    <t>unit type</t>
-  </si>
-  <si>
     <t>Descirbes the type of unit.</t>
   </si>
   <si>
-    <t>units delivered</t>
-  </si>
-  <si>
-    <t>units development</t>
-  </si>
-  <si>
     <t>Vintage</t>
   </si>
   <si>
@@ -228,13 +199,169 @@
   </si>
   <si>
     <t>Temporal period when the envrionmental benefit occurred</t>
+  </si>
+  <si>
+    <t>standard</t>
+  </si>
+  <si>
+    <t>American Carbon Registry (ACR) Standard</t>
+  </si>
+  <si>
+    <t>ERT</t>
+  </si>
+  <si>
+    <t>Emission Reduction Ton</t>
+  </si>
+  <si>
+    <t>ART-TREES Standard</t>
+  </si>
+  <si>
+    <t>TREES Credit</t>
+  </si>
+  <si>
+    <t>Bhutan's National Carbon Framework</t>
+  </si>
+  <si>
+    <t>BioCarbon Standard</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>Verified Carbon Credits</t>
+  </si>
+  <si>
+    <t>CAR Protocols</t>
+  </si>
+  <si>
+    <t>CRT</t>
+  </si>
+  <si>
+    <t>Climate Reserve Tonne</t>
+  </si>
+  <si>
+    <t>CDM Standard &amp; Methodologies</t>
+  </si>
+  <si>
+    <t>CER</t>
+  </si>
+  <si>
+    <t>Certified Emission Reduction</t>
+  </si>
+  <si>
+    <t>City Forests Credit (CFC) Standard</t>
+  </si>
+  <si>
+    <t>CFC</t>
+  </si>
+  <si>
+    <t>City Forest Carbon+ Credits</t>
+  </si>
+  <si>
+    <t>CNC Standard</t>
+  </si>
+  <si>
+    <t>Global Carbon Council Standard</t>
+  </si>
+  <si>
+    <t>ACC</t>
+  </si>
+  <si>
+    <t>Approved Carbon Credits</t>
+  </si>
+  <si>
+    <t>Gold Standard for the Global Goals</t>
+  </si>
+  <si>
+    <t>VER, CER</t>
+  </si>
+  <si>
+    <t>Voluntary Emission Reduction,Certified Emission Reduction</t>
+  </si>
+  <si>
+    <t>Isometric Standard</t>
+  </si>
+  <si>
+    <t>Isometric credit</t>
+  </si>
+  <si>
+    <t>JCM Standard</t>
+  </si>
+  <si>
+    <t>JCM Credits</t>
+  </si>
+  <si>
+    <t>Natural Forest Standard (NFS)</t>
+  </si>
+  <si>
+    <t>PACM Standard</t>
+  </si>
+  <si>
+    <t>A6.4 ER, MCU</t>
+  </si>
+  <si>
+    <t>Article 6.4 Emission Reductions, Mitigation Contribution Unit</t>
+  </si>
+  <si>
+    <t>Peatland Code</t>
+  </si>
+  <si>
+    <t>Plan Vivo Standard</t>
+  </si>
+  <si>
+    <t>PVC</t>
+  </si>
+  <si>
+    <t>Plan Vivo Certificates</t>
+  </si>
+  <si>
+    <t>Puro Standard</t>
+  </si>
+  <si>
+    <t>CORC</t>
+  </si>
+  <si>
+    <t>CO2 Removal Certificates</t>
+  </si>
+  <si>
+    <t>Verificed Carbon Standard (VCS)</t>
+  </si>
+  <si>
+    <t>VCU</t>
+  </si>
+  <si>
+    <t>Verified Carbon Unit</t>
+  </si>
+  <si>
+    <t>Woodland Carbon Code</t>
+  </si>
+  <si>
+    <t>PIU</t>
+  </si>
+  <si>
+    <t>Pre Issuance Unit</t>
+  </si>
+  <si>
+    <t>unit type short code</t>
+  </si>
+  <si>
+    <t>unit type name</t>
+  </si>
+  <si>
+    <t>JCM</t>
+  </si>
+  <si>
+    <t>status reason</t>
+  </si>
+  <si>
+    <t>type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -257,8 +384,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +409,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF073763"/>
+        <bgColor rgb="FF073763"/>
       </patternFill>
     </fill>
   </fills>
@@ -356,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -371,6 +517,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,7 +853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E3BF597-0DE1-7D40-BCE7-FF7BA286F3FE}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
@@ -745,471 +893,586 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="H2" s="7" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="G3" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>26</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="H7" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="H8" s="7" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>37</v>
+        <v>104</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>12</v>
-      </c>
       <c r="F10" s="5" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="G11" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="H12" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="H14" s="7" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="H15" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61BAD114-FACC-0146-B848-1E93BE75A30B}">
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" s="5" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="7" t="s">
+      <c r="B3" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+      <c r="C3" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>63</v>
-      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>